<commit_message>
Fix villa bedroom data and priceRange display for production
- Fixed 11 villas with incorrect bedroom/bathroom/guests data (Excel date serial numbers)
- Updated VillaCard to properly render priceRange object with display property
- Added /public/optimized-villas/ to .gitignore (850MB, using Cloudinary)
- Fixed TypeScript errors for production build
- Added VERCEL_ENV_SETUP.md with environment variables guide
- Removed unused imports (Phone, MessageCircle, CONTACT_INFO, usePathname)
- Build tested and passing successfully
</commit_message>
<xml_diff>
--- a/data/New EXVLSM Price Listing.xlsx
+++ b/data/New EXVLSM Price Listing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ronna\exclusive-villa-samui\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88CBA3DC-AA9E-475D-95D3-E8B77C438EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F81DA518-A3CA-4B46-AAA5-6F3C339DED4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4251,8 +4251,8 @@
     <col min="5" max="5" width="9.21875" customWidth="1"/>
     <col min="6" max="9" width="12.88671875" customWidth="1"/>
     <col min="10" max="10" width="54.44140625" customWidth="1"/>
-    <col min="11" max="11" width="15.88671875" customWidth="1"/>
-    <col min="12" max="12" width="15.44140625" customWidth="1"/>
+    <col min="11" max="11" width="26" customWidth="1"/>
+    <col min="12" max="12" width="26.77734375" customWidth="1"/>
     <col min="13" max="13" width="15.6640625" customWidth="1"/>
     <col min="14" max="14" width="16.33203125" customWidth="1"/>
     <col min="15" max="15" width="15.88671875" customWidth="1"/>
@@ -28221,5 +28221,6 @@
     <hyperlink ref="AH227" r:id="rId224" xr:uid="{00000000-0004-0000-0000-0000DF000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId225"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Switch to local storage image system - Update API endpoints to serve from database - Convert all image URLs to local paths - Add VillaImage model for professional image management - Ready for production deployment with 7,056 optimized images (850MB)
</commit_message>
<xml_diff>
--- a/data/New EXVLSM Price Listing.xlsx
+++ b/data/New EXVLSM Price Listing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ronna\exclusive-villa-samui\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F81DA518-A3CA-4B46-AAA5-6F3C339DED4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF6C6357-7730-48FE-8545-CAFE7A83FA0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3718,7 +3718,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3803,6 +3803,36 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor rgb="FFA4C2F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor rgb="FF3C78D8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -3831,7 +3861,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4023,6 +4053,35 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="5" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4377,7 +4436,7 @@
       </c>
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="84" t="s">
         <v>34</v>
       </c>
       <c r="B2" s="5" t="s">
@@ -10330,59 +10389,59 @@
       </c>
       <c r="AH95" s="19"/>
     </row>
-    <row r="96" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A96" s="20" t="s">
+    <row r="96" spans="1:34" s="81" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="74" t="s">
         <v>524</v>
       </c>
-      <c r="B96" s="20" t="s">
+      <c r="B96" s="74" t="s">
         <v>525</v>
       </c>
-      <c r="C96" s="20"/>
-      <c r="D96" s="9" t="s">
+      <c r="C96" s="74"/>
+      <c r="D96" s="75" t="s">
         <v>526</v>
       </c>
-      <c r="E96" s="44">
+      <c r="E96" s="76">
         <v>45844</v>
       </c>
-      <c r="F96" s="21" t="s">
+      <c r="F96" s="77" t="s">
         <v>520</v>
       </c>
-      <c r="G96" s="21" t="s">
+      <c r="G96" s="77" t="s">
         <v>37</v>
       </c>
-      <c r="H96" s="19" t="s">
+      <c r="H96" s="78" t="s">
         <v>371</v>
       </c>
-      <c r="I96" s="21"/>
-      <c r="J96" s="19" t="s">
+      <c r="I96" s="77"/>
+      <c r="J96" s="78" t="s">
         <v>521</v>
       </c>
-      <c r="K96" s="7" t="s">
+      <c r="K96" s="79" t="s">
         <v>522</v>
       </c>
-      <c r="L96" s="7"/>
-      <c r="M96" s="7"/>
-      <c r="N96" s="7"/>
-      <c r="O96" s="7"/>
-      <c r="P96" s="7"/>
-      <c r="Q96" s="7"/>
-      <c r="R96" s="7"/>
-      <c r="S96" s="7"/>
-      <c r="T96" s="7"/>
-      <c r="U96" s="7"/>
-      <c r="V96" s="7"/>
-      <c r="W96" s="8"/>
-      <c r="Z96" s="40"/>
-      <c r="AA96" s="40"/>
-      <c r="AB96" s="40"/>
-      <c r="AC96" s="40"/>
-      <c r="AD96" s="40"/>
-      <c r="AE96" s="40"/>
-      <c r="AF96" s="19"/>
-      <c r="AG96" s="30" t="s">
+      <c r="L96" s="79"/>
+      <c r="M96" s="79"/>
+      <c r="N96" s="79"/>
+      <c r="O96" s="79"/>
+      <c r="P96" s="79"/>
+      <c r="Q96" s="79"/>
+      <c r="R96" s="79"/>
+      <c r="S96" s="79"/>
+      <c r="T96" s="79"/>
+      <c r="U96" s="79"/>
+      <c r="V96" s="79"/>
+      <c r="W96" s="80"/>
+      <c r="Z96" s="82"/>
+      <c r="AA96" s="82"/>
+      <c r="AB96" s="82"/>
+      <c r="AC96" s="82"/>
+      <c r="AD96" s="82"/>
+      <c r="AE96" s="82"/>
+      <c r="AF96" s="78"/>
+      <c r="AG96" s="83" t="s">
         <v>523</v>
       </c>
-      <c r="AH96" s="19"/>
+      <c r="AH96" s="78"/>
     </row>
     <row r="97" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A97" s="20" t="s">

</xml_diff>